<commit_message>
feat: add new input excel version
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carlos/Desktop/script-cris-2024-05-22/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carlos/Desktop/Informatica/excel-transformer-script/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FBD8D13-2314-E740-85F1-A29724066E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2F6CE9-10B3-FD4C-BE14-99B9330D576A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-11620" yWindow="-28800" windowWidth="25480" windowHeight="28800" xr2:uid="{19895848-98C1-45AB-A46C-46A7D591448C}"/>
+    <workbookView xWindow="-11620" yWindow="-28800" windowWidth="51200" windowHeight="28800" xr2:uid="{19895848-98C1-45AB-A46C-46A7D591448C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$N$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
   <si>
     <t>FECHA ANÁLISIS</t>
   </si>
@@ -120,13 +120,19 @@
   </si>
   <si>
     <t>Column to not modify 3</t>
+  </si>
+  <si>
+    <t>Num events</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.000%"/>
+  </numFmts>
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -166,6 +172,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -258,7 +270,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -293,6 +305,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Entrada" xfId="1" builtinId="20"/>
@@ -314,9 +327,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -354,7 +367,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -460,7 +473,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -602,7 +615,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -613,24 +626,24 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="4" max="4" width="21" customWidth="1"/>
     <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="8" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="13.33203125" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -650,34 +663,37 @@
         <v>8</v>
       </c>
       <c r="G1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="M1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="N1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="O1" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="P1" s="7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
         <v>10</v>
       </c>
@@ -697,34 +713,38 @@
         <v>21</v>
       </c>
       <c r="G2">
+        <f>99*100 / 0.1</f>
+        <v>99000</v>
+      </c>
+      <c r="H2">
         <v>99</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>101</v>
       </c>
-      <c r="I2" s="8">
+      <c r="J2" s="8">
         <v>100</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>99</v>
       </c>
-      <c r="K2" s="9">
+      <c r="L2" s="9">
         <v>0.183</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <v>101</v>
       </c>
-      <c r="M2" s="9">
+      <c r="N2" s="9">
         <v>0.79500000000000004</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>100</v>
       </c>
-      <c r="O2" s="9">
+      <c r="P2" s="9">
         <v>0.79500000000000004</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>9</v>
       </c>
@@ -744,34 +764,37 @@
         <v>22</v>
       </c>
       <c r="G3">
-        <v>100</v>
+        <v>111111</v>
       </c>
       <c r="H3">
         <v>100</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3">
+        <v>100</v>
+      </c>
+      <c r="J3" s="8">
         <v>99</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>100</v>
       </c>
-      <c r="K3" s="9">
+      <c r="L3" s="9">
         <v>0.25600000000000001</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>100</v>
       </c>
-      <c r="M3" s="9">
+      <c r="N3" s="9">
         <v>0.71399999999999997</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>99</v>
       </c>
-      <c r="O3" s="9">
+      <c r="P3" s="9">
         <v>0.71399999999999997</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
         <v>11</v>
       </c>
@@ -791,42 +814,55 @@
         <v>23</v>
       </c>
       <c r="G4">
+        <v>91818</v>
+      </c>
+      <c r="H4">
         <v>101</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>99</v>
       </c>
-      <c r="I4" s="8">
+      <c r="J4" s="8">
         <v>101</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>101</v>
       </c>
-      <c r="K4" s="9">
+      <c r="L4" s="9">
         <v>0.30299999999999999</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <v>99</v>
       </c>
-      <c r="M4" s="9">
+      <c r="N4" s="9">
         <v>0.67100000000000004</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>101</v>
       </c>
-      <c r="O4" s="9">
+      <c r="P4" s="9">
         <v>0.67100000000000004</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="N6" s="10"/>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="O6" s="10"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="I15" s="14"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="I16" s="14"/>
+    </row>
+    <row r="17" spans="9:9" x14ac:dyDescent="0.2">
+      <c r="I17" s="14"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M1" xr:uid="{B3502221-9786-4040-B697-853A438B698C}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M9">
+  <autoFilter ref="A1:N1" xr:uid="{B3502221-9786-4040-B697-853A438B698C}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N9">
       <sortCondition descending="1" ref="D1:D9"/>
     </sortState>
   </autoFilter>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: add relative value strategy
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carlos/Desktop/Informatica/excel-transformer-script/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2F6CE9-10B3-FD4C-BE14-99B9330D576A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD012D89-16DF-DF4B-AAD2-1BE21BB8E295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-11620" yWindow="-28800" windowWidth="51200" windowHeight="28800" xr2:uid="{19895848-98C1-45AB-A46C-46A7D591448C}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{19895848-98C1-45AB-A46C-46A7D591448C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="2" r:id="rId1"/>
@@ -130,7 +130,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.000%"/>
+    <numFmt numFmtId="164" formatCode="0.000%"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -305,7 +305,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Entrada" xfId="1" builtinId="20"/>
@@ -713,7 +713,6 @@
         <v>21</v>
       </c>
       <c r="G2">
-        <f>99*100 / 0.1</f>
         <v>99000</v>
       </c>
       <c r="H2">

</xml_diff>

<commit_message>
style: input.xlsx - increase first row height
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carlos/Desktop/Informatica/excel-transformer-script/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD012D89-16DF-DF4B-AAD2-1BE21BB8E295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB06E823-AE85-D441-9879-467120110DAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{19895848-98C1-45AB-A46C-46A7D591448C}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16100" xr2:uid="{19895848-98C1-45AB-A46C-46A7D591448C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="2" r:id="rId1"/>
@@ -643,7 +643,7 @@
     <col min="16" max="16" width="14.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>